<commit_message>
Remove HeroLeague from project
</commit_message>
<xml_diff>
--- a/notebooks/URL_events.xlsx
+++ b/notebooks/URL_events.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keril\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyProjects\running-insights\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5D620D3-8B0C-4654-A56B-673863B46055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3F0D65-FCF6-4371-A0C8-A8EE2BFB8D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CA38AA2C-1D6F-4C6D-8A16-D354B1465C6C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="2026 год" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>